<commit_message>
7. multi truck import issue resolved
</commit_message>
<xml_diff>
--- a/rabbit-web-app/public/records/trailer_multi_services_bulk_sample.xlsx
+++ b/rabbit-web-app/public/records/trailer_multi_services_bulk_sample.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Bulk Multi-Services Trailers" sheetId="1" r:id="rId1"/>
+    <sheet name="Trailer Services" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,19 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="50.83203125" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="50.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:J6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,94 +442,94 @@
         <v>2026-08-19</v>
       </c>
       <c r="D2">
-        <v>1250</v>
+        <v>3200</v>
       </c>
       <c r="E2" t="str">
-        <v>90 Days inspection, Alignment, Alternator, Battery Change, Brakes, Grease, Hub Seal, Oil Change/Service</v>
+        <v>Annual Inspection</v>
       </c>
       <c r="F2" t="str">
-        <v>4th Axle (D/S), 5th Axle (P/S)</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>Hyundai Fleet Center</v>
+        <v>Utility Trailer Care</v>
       </c>
       <c r="H2" t="str">
-        <v>INV-TR-3001</v>
-      </c>
-      <c r="I2" t="str">
-        <v>1850.00</v>
+        <v>INV-TR-2001</v>
+      </c>
+      <c r="I2">
+        <v>1850</v>
       </c>
       <c r="J2" t="str">
-        <v>8-service maintenance with reefer unit and trailer brakes</v>
+        <v>Annual DOT inspection and trailer brake overhaul</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CH0014</v>
+        <v>BZ88BS77</v>
       </c>
       <c r="B3" t="str">
-        <v>DRY VAN</v>
+        <v>HYUNDAI</v>
       </c>
       <c r="C3" t="str">
         <v>2026-08-19</v>
       </c>
       <c r="D3">
-        <v>1180</v>
+        <v>3200</v>
       </c>
       <c r="E3" t="str">
-        <v>90 Days inspection, Alignment, Annual Inspection, Brakes, Bushing, Grease, Hub Seal, Oil Change/Service, Rotor, S-Cam, Shock, Slack Adjuster</v>
+        <v>Brakes</v>
       </c>
       <c r="F3" t="str">
-        <v>4th Axle (D/S), 4th Axle (P/S), 5th Axle (D/S)</v>
+        <v>4th Axle (D/S), 4th Axle (P/S)</v>
       </c>
       <c r="G3" t="str">
-        <v>National Trailer Hub</v>
+        <v>Utility Trailer Care</v>
       </c>
       <c r="H3" t="str">
-        <v>INV-TR-3002</v>
-      </c>
-      <c r="I3" t="str">
-        <v>3200.00</v>
+        <v>INV-TR-2001</v>
+      </c>
+      <c r="I3">
+        <v>1850</v>
       </c>
       <c r="J3" t="str">
-        <v>12-service brake &amp; suspension rebuild for Dry Van</v>
+        <v>Annual DOT inspection and trailer brake overhaul</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CH011</v>
+        <v>BZ88BS77</v>
       </c>
       <c r="B4" t="str">
-        <v>DRY VAN</v>
+        <v>HYUNDAI</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-18</v>
+        <v>2026-08-19</v>
       </c>
       <c r="D4">
-        <v>1320</v>
+        <v>3200</v>
       </c>
       <c r="E4" t="str">
-        <v>90 Days inspection, Alignment, Alternator, Annual Inspection, Battery Change, Grease, Hub Seal, Oil Change/Service, S-Cam, Slack Adjuster</v>
+        <v>Hub Seal</v>
       </c>
       <c r="F4" t="str">
-        <v>4th Axle (P/S), 5th Axle (D/S)</v>
+        <v>4th Axle (D/S), 5th Axle (P/S)</v>
       </c>
       <c r="G4" t="str">
-        <v>National Trailer Hub</v>
+        <v>Utility Trailer Care</v>
       </c>
       <c r="H4" t="str">
-        <v>INV-TR-3003</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2100.00</v>
+        <v>INV-TR-2001</v>
+      </c>
+      <c r="I4">
+        <v>1850</v>
       </c>
       <c r="J4" t="str">
-        <v>10-service inspection and S-Cam service</v>
+        <v>Annual DOT inspection and trailer brake overhaul</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CH012</v>
+        <v>TLR-902</v>
       </c>
       <c r="B5" t="str">
         <v>GREAT DANE</v>
@@ -550,190 +538,62 @@
         <v>2026-08-18</v>
       </c>
       <c r="D5">
-        <v>1290</v>
+        <v>2850</v>
       </c>
       <c r="E5" t="str">
-        <v>90 Days inspection, Alignment, Alternator, Annual Inspection, Battery Change, Brakes, Bushing, Grease, Hub Seal, Oil Change/Service, Rotor, S-Cam, Shock, Tires Change</v>
+        <v>Tires Change</v>
       </c>
       <c r="F5" t="str">
-        <v>4th Axle (D/S), 4th Axle (P/S), 5th Axle (D/S), 5th Axle (P/S)</v>
+        <v>4th Axle (D/S), 5th Axle (D/S)</v>
       </c>
       <c r="G5" t="str">
-        <v>Great Dane Fleet Care</v>
+        <v>Great Dane Hub</v>
       </c>
       <c r="H5" t="str">
-        <v>INV-TR-3004</v>
-      </c>
-      <c r="I5" t="str">
-        <v>4150.00</v>
+        <v>INV-TR-2002</v>
+      </c>
+      <c r="I5">
+        <v>2200</v>
       </c>
       <c r="J5" t="str">
-        <v>14-service full trailer overhaul including tire changes and rotors</v>
+        <v>Trailer tire replacement and alignment check</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>CH013</v>
+        <v>TLR-902</v>
       </c>
       <c r="B6" t="str">
-        <v>HYUNDAI</v>
+        <v>GREAT DANE</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-18</v>
       </c>
       <c r="D6">
-        <v>1140</v>
+        <v>2850</v>
       </c>
       <c r="E6" t="str">
-        <v>90 Days inspection, Alternator, Annual Inspection, Grease, Hub Seal, Oil Change/Service, Rotor, Slack Adjuster</v>
+        <v>Alignment</v>
       </c>
       <c r="F6" t="str">
-        <v>5th Axle (D/S), 5th Axle (P/S)</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>Hyundai Fleet Center</v>
+        <v>Great Dane Hub</v>
       </c>
       <c r="H6" t="str">
-        <v>INV-TR-3005</v>
-      </c>
-      <c r="I6" t="str">
-        <v>1920.00</v>
+        <v>INV-TR-2002</v>
+      </c>
+      <c r="I6">
+        <v>2200</v>
       </c>
       <c r="J6" t="str">
-        <v>8-service maintenance with rotor and slack adjuster replacement</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>CH016</v>
-      </c>
-      <c r="B7" t="str">
-        <v>HYUNDAI</v>
-      </c>
-      <c r="C7" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="D7">
-        <v>1420</v>
-      </c>
-      <c r="E7" t="str">
-        <v>90 Days inspection, Alignment, Alternator, Annual Inspection, Battery Change, Brakes, Bushing, Grease, Hub Seal, Oil Change/Service, S-Cam, Shock</v>
-      </c>
-      <c r="F7" t="str">
-        <v>4th Axle (D/S), 5th Axle (D/S)</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Speedy Trailer Service</v>
-      </c>
-      <c r="H7" t="str">
-        <v>INV-TR-3006</v>
-      </c>
-      <c r="I7" t="str">
-        <v>2850.00</v>
-      </c>
-      <c r="J7" t="str">
-        <v>12-service brake and shock replacement</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>CH017</v>
-      </c>
-      <c r="B8" t="str">
-        <v>HYUNDAI</v>
-      </c>
-      <c r="C8" t="str">
-        <v>2026-08-16</v>
-      </c>
-      <c r="D8">
-        <v>1380</v>
-      </c>
-      <c r="E8" t="str">
-        <v>90 Days inspection, Alignment, Alternator, Battery Change, Bushing, Grease, Hub Seal, Oil Change/Service, Shock, Starter</v>
-      </c>
-      <c r="F8" t="str">
-        <v>4th Axle (P/S), 5th Axle (D/S)</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Speedy Trailer Service</v>
-      </c>
-      <c r="H8" t="str">
-        <v>INV-TR-3007</v>
-      </c>
-      <c r="I8" t="str">
-        <v>2350.00</v>
-      </c>
-      <c r="J8" t="str">
-        <v>10-service reefer starter and bushing maintenance</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>CH018</v>
-      </c>
-      <c r="B9" t="str">
-        <v>HYUNDAI</v>
-      </c>
-      <c r="C9" t="str">
-        <v>2026-08-16</v>
-      </c>
-      <c r="D9">
-        <v>1310</v>
-      </c>
-      <c r="E9" t="str">
-        <v>90 Days inspection, Alignment, Alternator, Annual Inspection, Battery Change, Brakes, Bushing, Grease, Hub Seal, Oil Change/Service, Rotor, S-Cam, Slack Adjuster, Tires Change</v>
-      </c>
-      <c r="F9" t="str">
-        <v>4th Axle (D/S), 4th Axle (P/S), 5th Axle (D/S)</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Hyundai Fleet Center</v>
-      </c>
-      <c r="H9" t="str">
-        <v>INV-TR-3008</v>
-      </c>
-      <c r="I9" t="str">
-        <v>3950.00</v>
-      </c>
-      <c r="J9" t="str">
-        <v>14-service major maintenance including brakes and new tires</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>SMR2233</v>
-      </c>
-      <c r="B10" t="str">
-        <v>HYUNDAI</v>
-      </c>
-      <c r="C10" t="str">
-        <v>2026-08-15</v>
-      </c>
-      <c r="D10">
-        <v>1460</v>
-      </c>
-      <c r="E10" t="str">
-        <v>90 Days inspection, Alignment, Alternator, Annual Inspection, Battery Change, Brakes, Bushing, Grease, Hub Seal, Oil Change/Service, Rotor, S-Cam, Shock, Slack Adjuster, Tires Change, Water /Coolant Pump</v>
-      </c>
-      <c r="F10" t="str">
-        <v>4th Axle (D/S), 4th Axle (P/S), 5th Axle (D/S), 5th Axle (P/S)</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Apex Trailer Workshop</v>
-      </c>
-      <c r="H10" t="str">
-        <v>INV-TR-3009</v>
-      </c>
-      <c r="I10" t="str">
-        <v>4850.00</v>
-      </c>
-      <c r="J10" t="str">
-        <v>16-service full inspection, coolant pump, and complete brake kit</v>
+        <v>Trailer tire replacement and alignment check</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>